<commit_message>
Fix HTML report disclaimer and false RAG findings on clean samples
- Restore the Chinese "不构成法律意见" disclaimer and the
  "待外部复核字段清单" heading in the HTML report; re-add the test
  assertion that was dropped.
- Only the top-ranked matched template contributes required clauses, so a
  complaint is no longer held to the service-contract clause list.
- Give the synthetic KB client client-star-river-tech its own credit code
  and legal representative; it previously reused the identifiers of the
  legacy sample client, flagging clean samples as profile mismatches.
  Regenerate demo case files (demo-cases-v3) to match.
- Document the supported Python range (3.10-3.12) in README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_cases/files/clean_contract_pass/base_info.xlsx
+++ b/demo_cases/files/clean_contract_pass/base_info.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>张明远</t>
+          <t>沈牧舟</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>91310000MA1K000001</t>
+          <t>91310115MA1RXH0026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">

</xml_diff>